<commit_message>
Add KiCad files - schematic complete
</commit_message>
<xml_diff>
--- a/Bill of Materials.xlsx
+++ b/Bill of Materials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hardware\YieldGuard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C49E6C-2C1A-4054-A121-17052A7636ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9573E8-9240-41EA-96B3-A71D1E1CB7E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,9 +39,6 @@
     <t>Cost</t>
   </si>
   <si>
-    <t>ESP32-DevKitC V4 (38-Pin WROOM-32D Core)</t>
-  </si>
-  <si>
     <t>CZL-601 Aluminum Alloy 100kg Load Cell</t>
   </si>
   <si>
@@ -76,6 +73,9 @@
   </si>
   <si>
     <t>PCBWay</t>
+  </si>
+  <si>
+    <t>ESP32-DevKitC V4 ( WROOM-32D Core)</t>
   </si>
 </sst>
 </file>
@@ -136,7 +136,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -148,9 +148,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -459,13 +456,13 @@
     </row>
     <row r="4" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D4" s="1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E4" s="1">
         <v>1</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G4" s="3">
         <v>9.31</v>
@@ -473,13 +470,13 @@
     </row>
     <row r="5" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D5" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5" s="1">
         <v>1</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G5" s="3">
         <v>11.31</v>
@@ -487,13 +484,13 @@
     </row>
     <row r="6" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" s="1">
         <v>1</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G6" s="3">
         <v>1.89</v>
@@ -501,13 +498,13 @@
     </row>
     <row r="7" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="E7" s="1">
-        <v>1</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="G7" s="3">
         <v>0</v>
@@ -515,13 +512,13 @@
     </row>
     <row r="8" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D8" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E8" s="1">
         <v>1</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G8" s="3">
         <v>0</v>
@@ -529,13 +526,13 @@
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9" s="1">
         <v>1</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G9" s="3">
         <v>0</v>
@@ -543,13 +540,13 @@
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D10" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G10" s="3">
         <v>2</v>
@@ -557,18 +554,18 @@
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D11" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E11" s="1">
         <v>5</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>16</v>
+      <c r="F11" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D12" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>

</xml_diff>

<commit_message>
Bit changes in PCB and Schematic and Completed BoM
</commit_message>
<xml_diff>
--- a/Bill of Materials.xlsx
+++ b/Bill of Materials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hardware\YieldGuard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9573E8-9240-41EA-96B3-A71D1E1CB7E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B1DF486-24FD-47FD-B37E-E4C1B4765D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t>Item Name</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Micro-USB Cable</t>
   </si>
   <si>
-    <t>IP65 Waterproof Plastic Junction Box</t>
-  </si>
-  <si>
     <t>5V / 2A Phone Charger</t>
   </si>
   <si>
@@ -75,7 +72,16 @@
     <t>PCBWay</t>
   </si>
   <si>
-    <t>ESP32-DevKitC V4 ( WROOM-32D Core)</t>
+    <t>ESP32-C3-SuperMini</t>
+  </si>
+  <si>
+    <t>AliExpress Taxes</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>3D Case Shipping Charges</t>
   </si>
 </sst>
 </file>
@@ -136,7 +142,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -148,6 +154,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -456,7 +465,7 @@
     </row>
     <row r="4" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D4" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="1">
         <v>1</v>
@@ -465,7 +474,7 @@
         <v>13</v>
       </c>
       <c r="G4" s="3">
-        <v>9.31</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="5" spans="4:7" x14ac:dyDescent="0.3">
@@ -476,10 +485,10 @@
         <v>1</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" s="3">
-        <v>11.31</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="6" spans="4:7" x14ac:dyDescent="0.3">
@@ -493,7 +502,7 @@
         <v>13</v>
       </c>
       <c r="G6" s="3">
-        <v>1.89</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="7" spans="4:7" x14ac:dyDescent="0.3">
@@ -526,7 +535,7 @@
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D9" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E9" s="1">
         <v>1</v>
@@ -540,48 +549,55 @@
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D10" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>14</v>
+      <c r="F10" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="G10" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="1">
-        <v>5</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="3">
+        <v>7.6</v>
       </c>
     </row>
     <row r="12" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="1">
+        <v>5</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-    </row>
-    <row r="13" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-    </row>
-    <row r="14" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
+      <c r="G13" s="1">
+        <v>40</v>
+      </c>
     </row>
     <row r="15" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D15" s="1"/>
@@ -651,7 +667,6 @@
     <hyperlink ref="F4" r:id="rId1" xr:uid="{64852792-D8E1-4F25-90F6-404A09330F59}"/>
     <hyperlink ref="F5" r:id="rId2" xr:uid="{08E82361-03FF-4AE1-BC7C-9F8B240A7804}"/>
     <hyperlink ref="F6" r:id="rId3" xr:uid="{8B72833C-CB76-4A24-86AF-A6B1A9BF1E13}"/>
-    <hyperlink ref="F10" r:id="rId4" xr:uid="{C8873AB5-B42B-491B-8879-F60E5652E340}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>